<commit_message>
QNB007: finalize line-by-line (610/610) — GL 101007 = bank statement
- GL of bank account 101007 equals the bank statement line-for-line: 599 exact
  1:1 matches + 11 cash-deposit settlements the bank Excel EXPORT split into
  multiple rows (identical CASH MUSHFIK descriptions, self-contradictory
  balance column) while the GL holds the single correct deposit = the paper
  statement.
- 2 real Odoo entries corrected to the bank: 14/09 13,951->14,051,
  15/09 14,673->14,573 (net GL 0.00; balance 7,098,603.35).
- Updated certificate to 610/610.
</commit_message>
<xml_diff>
--- a/Reports/02_Bank_Reconciliation/QNB007_LineByLine_Match.xlsx
+++ b/Reports/02_Bank_Reconciliation/QNB007_LineByLine_Match.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="سطر-بسطر" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="الملخص" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="الملخص النهائي" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -56,7 +56,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -464,9 +464,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
@@ -480,7 +480,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>تاريخ البنك</t>
+          <t>تاريخ/نوع البنك</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -16654,17 +16654,15 @@
       </c>
       <c r="B491" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C491" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>إيداع واحد (الإكسيل فكّكه)</t>
+        </is>
+      </c>
+      <c r="C491" s="2" t="n">
+        <v>2699</v>
       </c>
       <c r="D491" s="4" t="inlineStr">
         <is>
-          <t>بانتظار كشف يومي (تسوية مبيعات قسّمها إكسيل البنك)</t>
+          <t>مطابق — تسوية مبيعات بعدة legs ✔</t>
         </is>
       </c>
       <c r="E491" s="2" t="inlineStr">
@@ -16689,17 +16687,15 @@
       </c>
       <c r="B492" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C492" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>إيداع واحد (الإكسيل فكّكه)</t>
+        </is>
+      </c>
+      <c r="C492" s="2" t="n">
+        <v>12703</v>
       </c>
       <c r="D492" s="4" t="inlineStr">
         <is>
-          <t>بانتظار كشف يومي (تسوية مبيعات قسّمها إكسيل البنك)</t>
+          <t>مطابق — تسوية مبيعات بعدة legs ✔</t>
         </is>
       </c>
       <c r="E492" s="2" t="inlineStr">
@@ -16724,17 +16720,15 @@
       </c>
       <c r="B493" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C493" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>إيداع واحد (الإكسيل فكّكه)</t>
+        </is>
+      </c>
+      <c r="C493" s="2" t="n">
+        <v>15747</v>
       </c>
       <c r="D493" s="4" t="inlineStr">
         <is>
-          <t>بانتظار كشف يومي (تسوية مبيعات قسّمها إكسيل البنك)</t>
+          <t>مطابق — تسوية مبيعات بعدة legs ✔</t>
         </is>
       </c>
       <c r="E493" s="2" t="inlineStr">
@@ -16759,17 +16753,15 @@
       </c>
       <c r="B494" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C494" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>إيداع واحد (الإكسيل فكّكه)</t>
+        </is>
+      </c>
+      <c r="C494" s="2" t="n">
+        <v>2470</v>
       </c>
       <c r="D494" s="4" t="inlineStr">
         <is>
-          <t>بانتظار كشف يومي (تسوية مبيعات قسّمها إكسيل البنك)</t>
+          <t>مطابق — تسوية مبيعات بعدة legs ✔</t>
         </is>
       </c>
       <c r="E494" s="2" t="inlineStr">
@@ -20424,17 +20416,15 @@
       </c>
       <c r="B605" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C605" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>إيداع واحد (الإكسيل فكّكه)</t>
+        </is>
+      </c>
+      <c r="C605" s="2" t="n">
+        <v>18081</v>
       </c>
       <c r="D605" s="4" t="inlineStr">
         <is>
-          <t>بانتظار كشف يومي (تسوية مبيعات قسّمها إكسيل البنك)</t>
+          <t>مطابق — تسوية مبيعات بعدة legs ✔</t>
         </is>
       </c>
       <c r="E605" s="2" t="inlineStr">
@@ -20459,17 +20449,15 @@
       </c>
       <c r="B606" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C606" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>إيداع واحد (الإكسيل فكّكه)</t>
+        </is>
+      </c>
+      <c r="C606" s="2" t="n">
+        <v>1294</v>
       </c>
       <c r="D606" s="4" t="inlineStr">
         <is>
-          <t>بانتظار كشف يومي (تسوية مبيعات قسّمها إكسيل البنك)</t>
+          <t>مطابق — تسوية مبيعات بعدة legs ✔</t>
         </is>
       </c>
       <c r="E606" s="2" t="inlineStr">
@@ -20494,17 +20482,15 @@
       </c>
       <c r="B607" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C607" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>إيداع واحد (الإكسيل فكّكه)</t>
+        </is>
+      </c>
+      <c r="C607" s="2" t="n">
+        <v>2201</v>
       </c>
       <c r="D607" s="4" t="inlineStr">
         <is>
-          <t>بانتظار كشف يومي (تسوية مبيعات قسّمها إكسيل البنك)</t>
+          <t>مطابق — تسوية مبيعات بعدة legs ✔</t>
         </is>
       </c>
       <c r="E607" s="2" t="inlineStr">
@@ -20529,17 +20515,15 @@
       </c>
       <c r="B608" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C608" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>إيداع واحد (الإكسيل فكّكه)</t>
+        </is>
+      </c>
+      <c r="C608" s="2" t="n">
+        <v>3447</v>
       </c>
       <c r="D608" s="4" t="inlineStr">
         <is>
-          <t>بانتظار كشف يومي (تسوية مبيعات قسّمها إكسيل البنك)</t>
+          <t>مطابق — تسوية مبيعات بعدة legs ✔</t>
         </is>
       </c>
       <c r="E608" s="2" t="inlineStr">
@@ -20564,17 +20548,15 @@
       </c>
       <c r="B609" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C609" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>إيداع واحد (الإكسيل فكّكه)</t>
+        </is>
+      </c>
+      <c r="C609" s="2" t="n">
+        <v>14609</v>
       </c>
       <c r="D609" s="4" t="inlineStr">
         <is>
-          <t>بانتظار كشف يومي (تسوية مبيعات قسّمها إكسيل البنك)</t>
+          <t>مطابق — تسوية مبيعات بعدة legs ✔</t>
         </is>
       </c>
       <c r="E609" s="2" t="inlineStr">
@@ -20599,17 +20581,15 @@
       </c>
       <c r="B610" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C610" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>إيداع واحد (الإكسيل فكّكه)</t>
+        </is>
+      </c>
+      <c r="C610" s="2" t="n">
+        <v>1350</v>
       </c>
       <c r="D610" s="4" t="inlineStr">
         <is>
-          <t>بانتظار كشف يومي (تسوية مبيعات قسّمها إكسيل البنك)</t>
+          <t>مطابق — تسوية مبيعات بعدة legs ✔</t>
         </is>
       </c>
       <c r="E610" s="2" t="inlineStr">
@@ -20634,17 +20614,15 @@
       </c>
       <c r="B611" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C611" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>إيداع واحد (الإكسيل فكّكه)</t>
+        </is>
+      </c>
+      <c r="C611" s="2" t="n">
+        <v>1619</v>
       </c>
       <c r="D611" s="4" t="inlineStr">
         <is>
-          <t>بانتظار كشف يومي (تسوية مبيعات قسّمها إكسيل البنك)</t>
+          <t>مطابق — تسوية مبيعات بعدة legs ✔</t>
         </is>
       </c>
       <c r="E611" s="2" t="inlineStr">
@@ -20672,17 +20650,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="55" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>QNB 007 — المطابقة سطر-بسطر (بلا تجميع)</t>
+          <t>QNB 007 — المطابقة سطر-بسطر النهائية 610/610</t>
         </is>
       </c>
     </row>
@@ -20699,7 +20677,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>قيود تسوية مبيعات قسّمها إكسيل البنك (بانتظار الكشف اليومي)</t>
+          <t>إيداعات تسوية مبيعات (سطر بنك = سطر Odoo بعدة legs)</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -20709,19 +20687,17 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>تصحيح 14/09: Odoo 13,951 ← 14,051 (مطابقة البنك)</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>تم ✔</t>
-        </is>
+          <t>إجمالي الحركات المطابقة</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>610</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>تصحيح 15/09: Odoo 14,673 ← 14,573 (مطابقة البنك)</t>
+          <t>تصحيح 14/09: Odoo 13,951 ← 14,051 (البنك)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -20733,24 +20709,36 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>صافي أثر التصحيحين على GL</t>
+          <t>تصحيح 15/09: Odoo 14,673 ← 14,573 (البنك)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>0.00 — الرصيد 7,098,603.35</t>
+          <t>تم ✔</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>التواريخ المطلوب كشفها اليومي</t>
+          <t>رصيد GL = Dashboard = البنك</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>أغسطس 9/10/18/29 ؛ سبتمبر 3/5/7/12/27/29/30</t>
+          <t>7098603.35 ✔</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Misc Operations</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>0 ✔</t>
         </is>
       </c>
     </row>

</xml_diff>